<commit_message>
Update: Tank Washouts fixed, conditioner additional rules
</commit_message>
<xml_diff>
--- a/APPT/data/output/Final_Production_Plan.xlsx
+++ b/APPT/data/output/Final_Production_Plan.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="371">
   <si>
     <t>Production Line</t>
   </si>
@@ -158,13 +158,31 @@
     <t>910731238 + 910731304</t>
   </si>
   <si>
-    <t>910728866 + 910728931 + 910728784 + 910728850</t>
+    <t>910731057</t>
+  </si>
+  <si>
+    <t>910728866 + 910728931</t>
+  </si>
+  <si>
+    <t>AUTO_1</t>
+  </si>
+  <si>
+    <t>910730961</t>
   </si>
   <si>
     <t>910728859</t>
   </si>
   <si>
-    <t>AUTO_1</t>
+    <t>910731220 + 910731319</t>
+  </si>
+  <si>
+    <t>910728784 + 910728850</t>
+  </si>
+  <si>
+    <t>910731210</t>
+  </si>
+  <si>
+    <t>910731292</t>
   </si>
   <si>
     <t>AUTO_2</t>
@@ -176,21 +194,6 @@
     <t>AUTO_3</t>
   </si>
   <si>
-    <t>910731057</t>
-  </si>
-  <si>
-    <t>910730961</t>
-  </si>
-  <si>
-    <t>910731220 + 910731319</t>
-  </si>
-  <si>
-    <t>910731210</t>
-  </si>
-  <si>
-    <t>910731292</t>
-  </si>
-  <si>
     <t>80880903</t>
   </si>
   <si>
@@ -227,33 +230,33 @@
     <t>80879278</t>
   </si>
   <si>
+    <t>80841060</t>
+  </si>
+  <si>
     <t>80841061</t>
   </si>
   <si>
+    <t>95619314</t>
+  </si>
+  <si>
+    <t>80851522</t>
+  </si>
+  <si>
     <t>83900258</t>
   </si>
   <si>
-    <t>95619314</t>
+    <t>80879275</t>
+  </si>
+  <si>
+    <t>80879287</t>
+  </si>
+  <si>
+    <t>80879283</t>
   </si>
   <si>
     <t>80880901</t>
   </si>
   <si>
-    <t>80841060</t>
-  </si>
-  <si>
-    <t>80851522</t>
-  </si>
-  <si>
-    <t>80879275</t>
-  </si>
-  <si>
-    <t>80879287</t>
-  </si>
-  <si>
-    <t>80879283</t>
-  </si>
-  <si>
     <t>H&amp;S SHM 180ML X 56 S&amp;S IN GST</t>
   </si>
   <si>
@@ -290,136 +293,139 @@
     <t>PNTN SHM 180MLX56 HS HFC IN GST</t>
   </si>
   <si>
+    <t>PNTN COND 200MLX 24 HS SS IN PC25</t>
+  </si>
+  <si>
     <t>PNTN COND 200MLX 24 HS HF IN PC25</t>
   </si>
   <si>
+    <t>Auto-Replenishment HC Base (12T)</t>
+  </si>
+  <si>
+    <t>PNTN COND 100MLX 24 HS HF IN AMJ25</t>
+  </si>
+  <si>
     <t>H&amp;S SHM 5.7MLX1200 NEEM IN GST FC</t>
   </si>
   <si>
-    <t>Auto-Replenishment HC Base (12T)</t>
+    <t>PNTN SHM 340ML X 30 HS LT IN GST</t>
+  </si>
+  <si>
+    <t>PNTN SHM 650ML X 12 HFC GST</t>
+  </si>
+  <si>
+    <t>PNTN SHM 650ML X 12 SSC IN GST</t>
   </si>
   <si>
     <t>H&amp;S SHM 180ML X 56 LF IN GST</t>
   </si>
   <si>
-    <t>PNTN COND 200MLX 24 HS SS IN PC25</t>
-  </si>
-  <si>
-    <t>PNTN COND 100MLX 24 HS HF IN AMJ25</t>
-  </si>
-  <si>
-    <t>PNTN SHM 340ML X 30 HS LT IN GST</t>
-  </si>
-  <si>
-    <t>PNTN SHM 650ML X 12 HFC GST</t>
-  </si>
-  <si>
-    <t>PNTN SHM 650ML X 12 SSC IN GST</t>
-  </si>
-  <si>
-    <t>B001</t>
-  </si>
-  <si>
     <t>B002</t>
   </si>
   <si>
+    <t>B003</t>
+  </si>
+  <si>
+    <t>B006</t>
+  </si>
+  <si>
+    <t>B007</t>
+  </si>
+  <si>
+    <t>B008</t>
+  </si>
+  <si>
+    <t>B010</t>
+  </si>
+  <si>
+    <t>B011</t>
+  </si>
+  <si>
+    <t>B012</t>
+  </si>
+  <si>
+    <t>B013</t>
+  </si>
+  <si>
+    <t>B014</t>
+  </si>
+  <si>
+    <t>B015</t>
+  </si>
+  <si>
+    <t>B016</t>
+  </si>
+  <si>
+    <t>B020</t>
+  </si>
+  <si>
+    <t>B021</t>
+  </si>
+  <si>
+    <t>B022</t>
+  </si>
+  <si>
+    <t>B023</t>
+  </si>
+  <si>
+    <t>B024</t>
+  </si>
+  <si>
+    <t>B025</t>
+  </si>
+  <si>
+    <t>B026</t>
+  </si>
+  <si>
+    <t>B027</t>
+  </si>
+  <si>
+    <t>B028</t>
+  </si>
+  <si>
+    <t>B029</t>
+  </si>
+  <si>
+    <t>B031</t>
+  </si>
+  <si>
+    <t>B032</t>
+  </si>
+  <si>
+    <t>B033</t>
+  </si>
+  <si>
+    <t>B004</t>
+  </si>
+  <si>
+    <t>REP01</t>
+  </si>
+  <si>
+    <t>B036</t>
+  </si>
+  <si>
     <t>B005</t>
   </si>
   <si>
-    <t>B006</t>
-  </si>
-  <si>
-    <t>B008</t>
-  </si>
-  <si>
-    <t>B009</t>
-  </si>
-  <si>
-    <t>B010</t>
-  </si>
-  <si>
-    <t>B011</t>
-  </si>
-  <si>
-    <t>B013</t>
-  </si>
-  <si>
-    <t>B014</t>
-  </si>
-  <si>
-    <t>B015</t>
-  </si>
-  <si>
-    <t>B016</t>
-  </si>
-  <si>
-    <t>B019</t>
-  </si>
-  <si>
-    <t>B020</t>
-  </si>
-  <si>
-    <t>B021</t>
-  </si>
-  <si>
-    <t>B022</t>
-  </si>
-  <si>
-    <t>B023</t>
-  </si>
-  <si>
-    <t>B024</t>
-  </si>
-  <si>
-    <t>B025</t>
-  </si>
-  <si>
-    <t>B026</t>
-  </si>
-  <si>
-    <t>B027</t>
-  </si>
-  <si>
-    <t>B028</t>
-  </si>
-  <si>
     <t>B030</t>
   </si>
   <si>
-    <t>B031</t>
-  </si>
-  <si>
-    <t>B003</t>
-  </si>
-  <si>
-    <t>B004</t>
-  </si>
-  <si>
-    <t>REP07</t>
-  </si>
-  <si>
-    <t>REP12</t>
+    <t>B018</t>
+  </si>
+  <si>
+    <t>B034</t>
+  </si>
+  <si>
+    <t>B035</t>
+  </si>
+  <si>
+    <t>REP09</t>
   </si>
   <si>
     <t>B017</t>
   </si>
   <si>
-    <t>REP18</t>
-  </si>
-  <si>
-    <t>B032</t>
-  </si>
-  <si>
-    <t>B035</t>
-  </si>
-  <si>
-    <t>B029</t>
-  </si>
-  <si>
-    <t>B033</t>
-  </si>
-  <si>
-    <t>B034</t>
+    <t>REP19</t>
   </si>
   <si>
     <t>21422079</t>
@@ -443,24 +449,24 @@
     <t>21302239</t>
   </si>
   <si>
+    <t>21090112</t>
+  </si>
+  <si>
     <t>21090111</t>
   </si>
   <si>
     <t>21448509</t>
   </si>
   <si>
+    <t>21302240</t>
+  </si>
+  <si>
+    <t>'21302240</t>
+  </si>
+  <si>
     <t>90966400</t>
   </si>
   <si>
-    <t>21090112</t>
-  </si>
-  <si>
-    <t>21302240</t>
-  </si>
-  <si>
-    <t>'21302240</t>
-  </si>
-  <si>
     <t>12T</t>
   </si>
   <si>
@@ -473,45 +479,126 @@
     <t>Dual</t>
   </si>
   <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>TK#_51_#</t>
-  </si>
-  <si>
-    <t>NO_TANK_AVAILABLE</t>
-  </si>
-  <si>
-    <t>TK#_22_#</t>
-  </si>
-  <si>
-    <t>TK#_16_#</t>
-  </si>
-  <si>
-    <t>TK#_12_#</t>
+    <t>TK#_51_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_7_# [Wash 20m] + TK#_6_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_23_# [Wash 20m] + TK#_24_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_21_# [Wash 20m] + TK#_2_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_17_# [Wash 20m] + TK#_20_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_3_# [Wash 20m] + TK#_4_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_1_# [Wash 20m] + TK#_18_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_13_# [Wash 20m] + TK#_7_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_6_# + TK#_19_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_16_# [Wash 20m] + TK#_15_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_23_# + TK#_24_#</t>
+  </si>
+  <si>
+    <t>TK#_8_# [Wash 20m] + TK#_21_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_17_# + TK#_20_#</t>
+  </si>
+  <si>
+    <t>TK#_52_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_53_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_6_# + TK#_19_#</t>
+  </si>
+  <si>
+    <t>TK#_22_# [Wash 20m] + TK#_5_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_1_# + TK#_18_#</t>
+  </si>
+  <si>
+    <t>TK#_52_#</t>
+  </si>
+  <si>
+    <t>TK#_27_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_26_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_17_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_25_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_13_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_11_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_28_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_10_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_9_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_8_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_5_# [Wash 20m]</t>
+  </si>
+  <si>
+    <t>TK#_22_# [Wash 20m]</t>
   </si>
   <si>
     <t>LOW: SLS</t>
   </si>
   <si>
+    <t>OK</t>
+  </si>
+  <si>
     <t>LOW: DM5500</t>
   </si>
   <si>
-    <t>OK</t>
-  </si>
-  <si>
     <t>Time</t>
   </si>
   <si>
     <t>1.25T</t>
   </si>
   <si>
+    <t>2026-01-13 07:30</t>
+  </si>
+  <si>
     <t>2026-01-13 08:00</t>
   </si>
   <si>
@@ -941,28 +1028,28 @@
     <t>2026-01-16 07:00</t>
   </si>
   <si>
-    <t>B001: H&amp;S SHM 180ML X 56 S&amp;S IN GST</t>
-  </si>
-  <si>
-    <t>B002: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
-  </si>
-  <si>
-    <t>B005: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
-  </si>
-  <si>
-    <t>B006: H&amp;S SHM 5.7MLX1200 DAILY COOL IN GST FC</t>
+    <t>B002: H&amp;S SHM 180ML X 56 S&amp;S IN GST</t>
+  </si>
+  <si>
+    <t>B003: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
+  </si>
+  <si>
+    <t>B006: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
+  </si>
+  <si>
+    <t>B007: H&amp;S SHM 5.7MLX1200 DAILY COOL IN GST FC</t>
   </si>
   <si>
     <t>B008: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
   </si>
   <si>
-    <t>B009: H&amp;S SHM 5.7MLX1200 DAILY COOL IN GST FC</t>
-  </si>
-  <si>
-    <t>B010: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
-  </si>
-  <si>
-    <t>B011: H&amp;S SHM 5.7MLX 960 DS IN GST FC</t>
+    <t>B010: H&amp;S SHM 5.7MLX1200 DAILY COOL IN GST FC</t>
+  </si>
+  <si>
+    <t>B011: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
+  </si>
+  <si>
+    <t>B012: H&amp;S SHM 5.7MLX 960 DS IN GST FC</t>
   </si>
   <si>
     <t>B013: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
@@ -977,79 +1064,70 @@
     <t>B016: H&amp;S SHM 180ML X 56 AHF IN GST</t>
   </si>
   <si>
+    <t>B020: H&amp;S SHM 5.7MLX1200 DS IN GST FC</t>
+  </si>
+  <si>
+    <t>B021: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
+  </si>
+  <si>
+    <t>B022: H&amp;S SHM 300ML X30 CM IN DM GST</t>
+  </si>
+  <si>
+    <t>B023: H&amp;S SHM 340ML X30 CM IN GST</t>
+  </si>
+  <si>
+    <t>B024: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
+  </si>
+  <si>
+    <t>B025: H&amp;S SHM 5.7MLX1200 DAILY CLEAN IN GST FC</t>
+  </si>
+  <si>
+    <t>B026: H&amp;S SHM 340ML X30 AHF IN GST</t>
+  </si>
+  <si>
+    <t>B027: PNTN SHM 340MLX30 HS HFC IN GST</t>
+  </si>
+  <si>
+    <t>B028: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
+  </si>
+  <si>
+    <t>B029: H&amp;S SHM 5.7MLX1200 DAILY CLEAN IN GST FC</t>
+  </si>
+  <si>
+    <t>B031: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
+  </si>
+  <si>
+    <t>B032: PNTN SHM 180MLX56 HS HFC IN GST</t>
+  </si>
+  <si>
+    <t>B033: PNTN COND 200MLX 24 HS SS IN PC25</t>
+  </si>
+  <si>
+    <t>B004: PNTN COND 200MLX 24 HS HF IN PC25</t>
+  </si>
+  <si>
+    <t>COND WASH (60m)</t>
+  </si>
+  <si>
+    <t>B036: PNTN COND 100MLX 24 HS HF IN AMJ25</t>
+  </si>
+  <si>
+    <t>B030: PNTN SHM 340ML X 30 HS LT IN GST</t>
+  </si>
+  <si>
     <t>WASHOUT</t>
   </si>
   <si>
-    <t>B019: H&amp;S SHM 5.7MLX1200 DS IN GST FC</t>
-  </si>
-  <si>
-    <t>B020: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
-  </si>
-  <si>
-    <t>B021: H&amp;S SHM 300ML X30 CM IN DM GST</t>
-  </si>
-  <si>
-    <t>B022: H&amp;S SHM 340ML X30 CM IN GST</t>
-  </si>
-  <si>
-    <t>B023: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
-  </si>
-  <si>
-    <t>B024: H&amp;S SHM 5.7MLX1200 DAILY CLEAN IN GST FC</t>
-  </si>
-  <si>
-    <t>B025: H&amp;S SHM 340ML X30 AHF IN GST</t>
-  </si>
-  <si>
-    <t>B026: PNTN SHM 340MLX30 HS HFC IN GST</t>
-  </si>
-  <si>
-    <t>B027: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
-  </si>
-  <si>
-    <t>B028: H&amp;S SHM 5.7MLX1200 DAILY CLEAN IN GST FC</t>
-  </si>
-  <si>
-    <t>B030: H&amp;S SHM 5.7MLX960 DAILY CLEAN IN GST FC</t>
-  </si>
-  <si>
-    <t>B031: PNTN SHM 180MLX56 HS HFC IN GST</t>
-  </si>
-  <si>
-    <t>B003: PNTN COND 200MLX 24 HS HF IN PC25</t>
-  </si>
-  <si>
-    <t>COND WASH (60m)</t>
-  </si>
-  <si>
-    <t>B004: H&amp;S SHM 5.7MLX1200 NEEM IN GST FC</t>
-  </si>
-  <si>
-    <t>REP07: Auto-Replenishment HC Base (12T)</t>
-  </si>
-  <si>
-    <t>REP12: Auto-Replenishment HC Base (12T)</t>
+    <t>B034: PNTN SHM 650ML X 12 HFC GST</t>
+  </si>
+  <si>
+    <t>REP09: Auto-Replenishment HC Base (12T)</t>
   </si>
   <si>
     <t>B017: H&amp;S SHM 180ML X 56 LF IN GST</t>
   </si>
   <si>
-    <t>REP18: Auto-Replenishment HC Base (12T)</t>
-  </si>
-  <si>
-    <t>B032: PNTN COND 200MLX 24 HS SS IN PC25</t>
-  </si>
-  <si>
-    <t>B035: PNTN COND 100MLX 24 HS HF IN AMJ25</t>
-  </si>
-  <si>
-    <t>B029: PNTN SHM 340ML X 30 HS LT IN GST</t>
-  </si>
-  <si>
-    <t>B033: PNTN SHM 650ML X 12 HFC GST</t>
-  </si>
-  <si>
-    <t>B034: PNTN SHM 650ML X 12 SSC IN GST</t>
+    <t>REP19: Auto-Replenishment HC Base (12T)</t>
   </si>
 </sst>
 </file>
@@ -1411,7 +1489,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R36"/>
+  <dimension ref="A1:R37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="18" width="15.7109375" customWidth="1"/>
@@ -1481,43 +1559,43 @@
         <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H2">
         <v>4.5088</v>
       </c>
       <c r="I2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="K2" s="2">
-        <v>46036.16041666667</v>
+        <v>46035.72916666666</v>
       </c>
       <c r="L2">
         <v>90</v>
       </c>
       <c r="M2" s="2">
-        <v>46036.22291666667</v>
+        <v>46035.79166666666</v>
       </c>
       <c r="N2">
-        <v>199</v>
+        <v>820</v>
       </c>
       <c r="O2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="P2" s="2">
         <v>46036.36111111111</v>
@@ -1526,7 +1604,7 @@
         <v>46036.55</v>
       </c>
       <c r="R2" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -1537,43 +1615,43 @@
         <v>24</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H3">
         <v>4.4185</v>
       </c>
       <c r="I3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="K3" s="2">
-        <v>46036.22291666667</v>
+        <v>46035.79166666666</v>
       </c>
       <c r="L3">
         <v>90</v>
       </c>
       <c r="M3" s="2">
-        <v>46036.28541666667</v>
+        <v>46035.85416666666</v>
       </c>
       <c r="N3">
-        <v>120</v>
+        <v>741</v>
       </c>
       <c r="O3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="P3" s="2">
         <v>46036.36875</v>
@@ -1582,7 +1660,7 @@
         <v>46036.55208333334</v>
       </c>
       <c r="R3" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -1593,43 +1671,43 @@
         <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F4" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G4" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H4">
         <v>4.4185</v>
       </c>
       <c r="I4" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K4" s="2">
-        <v>46036.35902777778</v>
+        <v>46035.85416666666</v>
       </c>
       <c r="L4">
         <v>90</v>
       </c>
       <c r="M4" s="2">
-        <v>46036.42152777778</v>
+        <v>46035.91666666666</v>
       </c>
       <c r="N4">
-        <v>188</v>
+        <v>915</v>
       </c>
       <c r="O4" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="P4" s="2">
         <v>46036.55208333334</v>
@@ -1638,7 +1716,7 @@
         <v>46036.73611111111</v>
       </c>
       <c r="R4" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" spans="1:18">
@@ -1649,43 +1727,43 @@
         <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H5">
         <v>4.4163</v>
       </c>
       <c r="I5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K5" s="2">
-        <v>46036.42152777778</v>
+        <v>46035.91666666666</v>
       </c>
       <c r="L5">
         <v>90</v>
       </c>
       <c r="M5" s="2">
-        <v>46036.48402777778</v>
+        <v>46035.97916666666</v>
       </c>
       <c r="N5">
-        <v>120</v>
+        <v>847</v>
       </c>
       <c r="O5" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="P5" s="2">
         <v>46036.56736111111</v>
@@ -1694,7 +1772,7 @@
         <v>46036.78125</v>
       </c>
       <c r="R5" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="6" spans="1:18">
@@ -1705,43 +1783,43 @@
         <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H6">
         <v>4.4185</v>
       </c>
       <c r="I6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K6" s="2">
-        <v>46036.59027777778</v>
+        <v>46036.34027777778</v>
       </c>
       <c r="L6">
         <v>90</v>
       </c>
       <c r="M6" s="2">
-        <v>46036.65277777778</v>
+        <v>46036.40277777778</v>
       </c>
       <c r="N6">
-        <v>120</v>
+        <v>480</v>
       </c>
       <c r="O6" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="P6" s="2">
         <v>46036.73611111111</v>
@@ -1750,7 +1828,7 @@
         <v>46036.91944444444</v>
       </c>
       <c r="R6" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="7" spans="1:18">
@@ -1761,43 +1839,43 @@
         <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F7" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H7">
         <v>4.4163</v>
       </c>
       <c r="I7" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K7" s="2">
-        <v>46036.67708333334</v>
+        <v>46036.40277777778</v>
       </c>
       <c r="L7">
         <v>90</v>
       </c>
       <c r="M7" s="2">
-        <v>46036.73958333334</v>
+        <v>46036.46527777778</v>
       </c>
       <c r="N7">
-        <v>120</v>
+        <v>515</v>
       </c>
       <c r="O7" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="P7" s="2">
         <v>46036.82291666666</v>
@@ -1806,7 +1884,7 @@
         <v>46037.03611111111</v>
       </c>
       <c r="R7" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" spans="1:18">
@@ -1817,43 +1895,43 @@
         <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F8" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G8" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H8">
         <v>4.4185</v>
       </c>
       <c r="I8" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K8" s="2">
-        <v>46036.77361111111</v>
+        <v>46036.46527777778</v>
       </c>
       <c r="L8">
         <v>90</v>
       </c>
       <c r="M8" s="2">
-        <v>46036.83611111111</v>
+        <v>46036.52777777778</v>
       </c>
       <c r="N8">
-        <v>120</v>
+        <v>564</v>
       </c>
       <c r="O8" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="P8" s="2">
         <v>46036.91944444444</v>
@@ -1862,7 +1940,7 @@
         <v>46037.10347222222</v>
       </c>
       <c r="R8" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="9" spans="1:18">
@@ -1873,43 +1951,43 @@
         <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F9" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G9" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H9">
         <v>4.4185</v>
       </c>
       <c r="I9" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J9" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K9" s="2">
-        <v>46036.84166666667</v>
+        <v>46036.52777777778</v>
       </c>
       <c r="L9">
         <v>90</v>
       </c>
       <c r="M9" s="2">
-        <v>46036.90416666667</v>
+        <v>46036.59027777778</v>
       </c>
       <c r="N9">
-        <v>190</v>
+        <v>642</v>
       </c>
       <c r="O9" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="P9" s="2">
         <v>46037.03611111111</v>
@@ -1918,7 +1996,7 @@
         <v>46037.25</v>
       </c>
       <c r="R9" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="10" spans="1:18">
@@ -1929,43 +2007,43 @@
         <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G10" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H10">
         <v>4.4185</v>
       </c>
       <c r="I10" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J10" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K10" s="2">
-        <v>46036.90416666667</v>
+        <v>46036.59027777778</v>
       </c>
       <c r="L10">
         <v>90</v>
       </c>
       <c r="M10" s="2">
-        <v>46036.96666666667</v>
+        <v>46036.65277777778</v>
       </c>
       <c r="N10">
-        <v>197</v>
+        <v>649</v>
       </c>
       <c r="O10" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="P10" s="2">
         <v>46037.10347222222</v>
@@ -1974,7 +2052,7 @@
         <v>46037.28680555556</v>
       </c>
       <c r="R10" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="11" spans="1:18">
@@ -1985,43 +2063,43 @@
         <v>32</v>
       </c>
       <c r="C11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D11" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F11" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H11">
         <v>4.4185</v>
       </c>
       <c r="I11" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J11" t="s">
         <v>154</v>
       </c>
       <c r="K11" s="2">
-        <v>46036.96666666667</v>
+        <v>46036.65277777778</v>
       </c>
       <c r="L11">
         <v>90</v>
       </c>
       <c r="M11" s="2">
-        <v>46037.02916666667</v>
+        <v>46036.71527777778</v>
       </c>
       <c r="N11">
-        <v>318</v>
+        <v>770</v>
       </c>
       <c r="O11" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="P11" s="2">
         <v>46037.25</v>
@@ -2030,7 +2108,7 @@
         <v>46037.46319444444</v>
       </c>
       <c r="R11" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="12" spans="1:18">
@@ -2041,43 +2119,43 @@
         <v>33</v>
       </c>
       <c r="C12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G12" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H12">
         <v>4.4185</v>
       </c>
       <c r="I12" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J12" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="K12" s="2">
-        <v>46037.02916666667</v>
+        <v>46036.71527777778</v>
       </c>
       <c r="L12">
         <v>90</v>
       </c>
       <c r="M12" s="2">
-        <v>46037.09166666667</v>
+        <v>46036.77777777778</v>
       </c>
       <c r="N12">
-        <v>281</v>
+        <v>733</v>
       </c>
       <c r="O12" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="P12" s="2">
         <v>46037.28680555556</v>
@@ -2086,7 +2164,7 @@
         <v>46037.47083333333</v>
       </c>
       <c r="R12" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="13" spans="1:18">
@@ -2097,43 +2175,43 @@
         <v>34</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F13" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G13" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H13">
         <v>4.4891</v>
       </c>
       <c r="I13" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="K13" s="2">
-        <v>46037.09166666667</v>
+        <v>46036.77777777778</v>
       </c>
       <c r="L13">
         <v>90</v>
       </c>
       <c r="M13" s="2">
-        <v>46037.15416666667</v>
+        <v>46036.84027777778</v>
       </c>
       <c r="N13">
-        <v>228</v>
+        <v>680</v>
       </c>
       <c r="O13" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="P13" s="2">
         <v>46037.3125</v>
@@ -2142,7 +2220,7 @@
         <v>46037.75833333333</v>
       </c>
       <c r="R13" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="14" spans="1:18">
@@ -2153,43 +2231,43 @@
         <v>35</v>
       </c>
       <c r="C14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F14" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G14" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H14">
         <v>4.4163</v>
       </c>
       <c r="I14" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J14" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="K14" s="2">
-        <v>46037.16805555556</v>
+        <v>46036.85416666666</v>
       </c>
       <c r="L14">
         <v>90</v>
       </c>
       <c r="M14" s="2">
-        <v>46037.23055555556</v>
+        <v>46036.91666666666</v>
       </c>
       <c r="N14">
-        <v>335</v>
+        <v>787</v>
       </c>
       <c r="O14" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="P14" s="2">
         <v>46037.46319444444</v>
@@ -2198,7 +2276,7 @@
         <v>46037.67708333334</v>
       </c>
       <c r="R14" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="15" spans="1:18">
@@ -2209,43 +2287,43 @@
         <v>36</v>
       </c>
       <c r="C15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F15" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G15" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H15">
         <v>4.4185</v>
       </c>
       <c r="I15" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J15" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="K15" s="2">
-        <v>46037.23055555556</v>
+        <v>46036.91666666666</v>
       </c>
       <c r="L15">
         <v>90</v>
       </c>
       <c r="M15" s="2">
-        <v>46037.29305555556</v>
+        <v>46036.97916666666</v>
       </c>
       <c r="N15">
-        <v>256</v>
+        <v>708</v>
       </c>
       <c r="O15" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="P15" s="2">
         <v>46037.47083333333</v>
@@ -2254,7 +2332,7 @@
         <v>46037.65486111111</v>
       </c>
       <c r="R15" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="16" spans="1:18">
@@ -2265,28 +2343,28 @@
         <v>37</v>
       </c>
       <c r="C16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F16" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="G16" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H16">
         <v>4.0957</v>
       </c>
       <c r="I16" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J16" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="K16" s="2">
         <v>46037.29305555556</v>
@@ -2301,7 +2379,7 @@
         <v>209</v>
       </c>
       <c r="O16" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="P16" s="2">
         <v>46037.50069444445</v>
@@ -2310,7 +2388,7 @@
         <v>46037.6375</v>
       </c>
       <c r="R16" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="17" spans="1:18">
@@ -2321,28 +2399,28 @@
         <v>38</v>
       </c>
       <c r="C17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D17" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E17" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F17" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="G17" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H17">
         <v>5.2051</v>
       </c>
       <c r="I17" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J17" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K17" s="2">
         <v>46037.35555555556</v>
@@ -2357,7 +2435,7 @@
         <v>316</v>
       </c>
       <c r="O17" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="P17" s="2">
         <v>46037.6375</v>
@@ -2366,7 +2444,7 @@
         <v>46038.77569444444</v>
       </c>
       <c r="R17" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="18" spans="1:18">
@@ -2377,28 +2455,28 @@
         <v>39</v>
       </c>
       <c r="C18" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F18" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G18" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H18">
         <v>4.4185</v>
       </c>
       <c r="I18" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J18" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K18" s="2">
         <v>46037.41805555556</v>
@@ -2413,7 +2491,7 @@
         <v>251</v>
       </c>
       <c r="O18" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="P18" s="2">
         <v>46037.65486111111</v>
@@ -2422,7 +2500,7 @@
         <v>46037.83819444444</v>
       </c>
       <c r="R18" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="19" spans="1:18">
@@ -2433,28 +2511,28 @@
         <v>40</v>
       </c>
       <c r="C19" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D19" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F19" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G19" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H19">
         <v>4.4163</v>
       </c>
       <c r="I19" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J19" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K19" s="2">
         <v>46037.48055555556</v>
@@ -2469,7 +2547,7 @@
         <v>193</v>
       </c>
       <c r="O19" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
       <c r="P19" s="2">
         <v>46037.67708333334</v>
@@ -2478,7 +2556,7 @@
         <v>46037.89027777778</v>
       </c>
       <c r="R19" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="20" spans="1:18">
@@ -2489,28 +2567,28 @@
         <v>41</v>
       </c>
       <c r="C20" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D20" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F20" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G20" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H20">
         <v>5.2051</v>
       </c>
       <c r="I20" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J20" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K20" s="2">
         <v>46037.54305555556</v>
@@ -2525,7 +2603,7 @@
         <v>220</v>
       </c>
       <c r="O20" t="s">
-        <v>156</v>
+        <v>173</v>
       </c>
       <c r="P20" s="2">
         <v>46037.75833333333</v>
@@ -2534,7 +2612,7 @@
         <v>46038.71527777778</v>
       </c>
       <c r="R20" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="21" spans="1:18">
@@ -2545,28 +2623,28 @@
         <v>42</v>
       </c>
       <c r="C21" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D21" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F21" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G21" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H21">
         <v>4.5228</v>
       </c>
       <c r="I21" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="J21" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K21" s="2">
         <v>46037.61944444444</v>
@@ -2581,7 +2659,7 @@
         <v>196</v>
       </c>
       <c r="O21" t="s">
-        <v>155</v>
+        <v>170</v>
       </c>
       <c r="P21" s="2">
         <v>46037.81805555556</v>
@@ -2590,7 +2668,7 @@
         <v>46037.93819444445</v>
       </c>
       <c r="R21" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="22" spans="1:18">
@@ -2601,25 +2679,25 @@
         <v>43</v>
       </c>
       <c r="C22" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D22" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F22" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H22">
         <v>4.4185</v>
       </c>
       <c r="I22" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J22" t="s">
         <v>154</v>
@@ -2637,7 +2715,7 @@
         <v>135</v>
       </c>
       <c r="O22" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="P22" s="2">
         <v>46037.83819444444</v>
@@ -2646,7 +2724,7 @@
         <v>46038.02222222222</v>
       </c>
       <c r="R22" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="23" spans="1:18">
@@ -2657,25 +2735,25 @@
         <v>44</v>
       </c>
       <c r="C23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D23" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E23" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F23" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G23" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H23">
         <v>4.4163</v>
       </c>
       <c r="I23" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J23" t="s">
         <v>154</v>
@@ -2693,7 +2771,7 @@
         <v>120</v>
       </c>
       <c r="O23" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
       <c r="P23" s="2">
         <v>46037.89027777778</v>
@@ -2702,7 +2780,7 @@
         <v>46038.10416666666</v>
       </c>
       <c r="R23" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="24" spans="1:18">
@@ -2713,25 +2791,25 @@
         <v>45</v>
       </c>
       <c r="C24" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D24" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F24" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G24" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H24">
         <v>4.4185</v>
       </c>
       <c r="I24" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J24" t="s">
         <v>154</v>
@@ -2749,7 +2827,7 @@
         <v>120</v>
       </c>
       <c r="O24" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
       <c r="P24" s="2">
         <v>46038.02222222222</v>
@@ -2758,7 +2836,7 @@
         <v>46038.20555555556</v>
       </c>
       <c r="R24" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="25" spans="1:18">
@@ -2769,28 +2847,28 @@
         <v>46</v>
       </c>
       <c r="C25" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D25" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F25" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G25" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H25">
         <v>5.1635</v>
       </c>
       <c r="I25" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="J25" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="K25" s="2">
         <v>46038.23472222222</v>
@@ -2805,7 +2883,7 @@
         <v>120</v>
       </c>
       <c r="O25" t="s">
-        <v>155</v>
+        <v>175</v>
       </c>
       <c r="P25" s="2">
         <v>46038.38055555556</v>
@@ -2814,7 +2892,7 @@
         <v>46038.53472222222</v>
       </c>
       <c r="R25" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="26" spans="1:18">
@@ -2825,108 +2903,108 @@
         <v>47</v>
       </c>
       <c r="C26" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F26" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G26" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H26">
-        <v>2.2404</v>
+        <v>0.5601</v>
       </c>
       <c r="I26" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J26" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K26" s="2">
-        <v>46035.33333333334</v>
+        <v>46035.3125</v>
       </c>
       <c r="L26">
         <v>90</v>
       </c>
       <c r="M26" s="2">
-        <v>46035.39583333334</v>
+        <v>46035.375</v>
       </c>
       <c r="N26">
-        <v>1440</v>
+        <v>4393</v>
       </c>
       <c r="O26" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="P26" s="2">
-        <v>46036.39583333334</v>
+        <v>46038.42569444444</v>
       </c>
       <c r="Q26" s="2">
-        <v>46038.42569444444</v>
+        <v>46038.60486111111</v>
       </c>
       <c r="R26" t="s">
-        <v>161</v>
+        <v>189</v>
       </c>
     </row>
     <row r="27" spans="1:18">
       <c r="A27" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B27" t="s">
         <v>48</v>
       </c>
       <c r="C27" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D27" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E27" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F27" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G27" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H27">
-        <v>2.2082</v>
+        <v>1.1202</v>
       </c>
       <c r="I27" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J27" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K27" s="2">
-        <v>46035.4375</v>
+        <v>46035.33333333334</v>
       </c>
       <c r="L27">
         <v>90</v>
       </c>
       <c r="M27" s="2">
-        <v>46035.5</v>
+        <v>46035.39583333334</v>
       </c>
       <c r="N27">
-        <v>1384</v>
+        <v>1440</v>
       </c>
       <c r="O27" t="s">
-        <v>158</v>
+        <v>177</v>
       </c>
       <c r="P27" s="2">
-        <v>46036.46111111111</v>
+        <v>46036.39583333334</v>
       </c>
       <c r="Q27" s="2">
-        <v>46036.56736111111</v>
+        <v>46037.41041666667</v>
       </c>
       <c r="R27" t="s">
-        <v>160</v>
+        <v>190</v>
       </c>
     </row>
     <row r="28" spans="1:18">
@@ -2937,220 +3015,220 @@
         <v>49</v>
       </c>
       <c r="C28" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D28" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E28" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F28" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G28" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H28">
         <v>2.2948</v>
       </c>
       <c r="I28" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J28" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K28" s="2">
-        <v>46035.51388888889</v>
+        <v>46035.4375</v>
       </c>
       <c r="L28">
         <v>90</v>
       </c>
       <c r="M28" s="2">
-        <v>46035.57638888889</v>
+        <v>46035.5</v>
       </c>
       <c r="N28">
-        <v>1430</v>
+        <v>1180</v>
       </c>
       <c r="O28" t="s">
-        <v>159</v>
+        <v>178</v>
       </c>
       <c r="P28" s="2">
-        <v>46036.56944444445</v>
+        <v>46036.31944444445</v>
       </c>
       <c r="Q28" s="2">
-        <v>46036.61111111111</v>
+        <v>46036.36111111111</v>
       </c>
       <c r="R28" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="29" spans="1:18">
       <c r="A29" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B29" t="s">
         <v>50</v>
       </c>
       <c r="C29" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D29" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E29" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F29" t="s">
-        <v>72</v>
+        <v>145</v>
       </c>
       <c r="G29" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H29">
-        <v>2.2948</v>
+        <v>0.28</v>
       </c>
       <c r="I29" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J29" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K29" s="2">
-        <v>46035.57638888889</v>
+        <v>46035.4375</v>
       </c>
       <c r="L29">
         <v>90</v>
       </c>
       <c r="M29" s="2">
-        <v>46035.63888888889</v>
+        <v>46035.5</v>
       </c>
       <c r="N29">
-        <v>2062</v>
+        <v>4471</v>
       </c>
       <c r="O29" t="s">
-        <v>156</v>
+        <v>179</v>
       </c>
       <c r="P29" s="2">
-        <v>46037.07083333333</v>
+        <v>46038.60486111111</v>
       </c>
       <c r="Q29" s="2">
-        <v>46037.1125</v>
+        <v>46039.42569444444</v>
       </c>
       <c r="R29" t="s">
-        <v>160</v>
+        <v>190</v>
       </c>
     </row>
     <row r="30" spans="1:18">
       <c r="A30" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B30" t="s">
         <v>51</v>
       </c>
       <c r="C30" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D30" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F30" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G30" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H30">
-        <v>2.2544</v>
+        <v>2.2082</v>
       </c>
       <c r="I30" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J30" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K30" s="2">
-        <v>46035.65277777778</v>
+        <v>46035.51388888889</v>
       </c>
       <c r="L30">
         <v>90</v>
       </c>
       <c r="M30" s="2">
-        <v>46035.71527777778</v>
+        <v>46035.57638888889</v>
       </c>
       <c r="N30">
-        <v>2435</v>
+        <v>1274</v>
       </c>
       <c r="O30" t="s">
-        <v>156</v>
+        <v>180</v>
       </c>
       <c r="P30" s="2">
-        <v>46037.40625</v>
+        <v>46036.46111111111</v>
       </c>
       <c r="Q30" s="2">
-        <v>46037.50069444445</v>
+        <v>46036.56736111111</v>
       </c>
       <c r="R30" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="31" spans="1:18">
       <c r="A31" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B31" t="s">
         <v>52</v>
       </c>
       <c r="C31" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D31" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="E31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F31" t="s">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="G31" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H31">
-        <v>2.2948</v>
+        <v>2.2733</v>
       </c>
       <c r="I31" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J31" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K31" s="2">
-        <v>46035.72916666666</v>
+        <v>46035.54166666666</v>
       </c>
       <c r="L31">
         <v>90</v>
       </c>
       <c r="M31" s="2">
-        <v>46035.79166666666</v>
+        <v>46035.60416666666</v>
       </c>
       <c r="N31">
-        <v>2402</v>
+        <v>3361</v>
       </c>
       <c r="O31" t="s">
-        <v>156</v>
+        <v>181</v>
       </c>
       <c r="P31" s="2">
-        <v>46037.45972222222</v>
+        <v>46037.93819444445</v>
       </c>
       <c r="Q31" s="2">
-        <v>46037.50138888889</v>
+        <v>46038.38055555556</v>
       </c>
       <c r="R31" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="32" spans="1:18">
@@ -3161,108 +3239,108 @@
         <v>53</v>
       </c>
       <c r="C32" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D32" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E32" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F32" t="s">
         <v>145</v>
       </c>
       <c r="G32" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H32">
-        <v>0.5601</v>
+        <v>1.1202</v>
       </c>
       <c r="I32" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J32" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K32" s="2">
-        <v>46035.82638888889</v>
+        <v>46035.61111111111</v>
       </c>
       <c r="L32">
         <v>90</v>
       </c>
       <c r="M32" s="2">
-        <v>46035.88888888889</v>
+        <v>46035.67361111111</v>
       </c>
       <c r="N32">
-        <v>3653</v>
+        <v>2501</v>
       </c>
       <c r="O32" t="s">
-        <v>156</v>
+        <v>182</v>
       </c>
       <c r="P32" s="2">
+        <v>46037.41041666667</v>
+      </c>
+      <c r="Q32" s="2">
         <v>46038.42569444444</v>
       </c>
-      <c r="Q32" s="2">
-        <v>46038.60486111111</v>
-      </c>
       <c r="R32" t="s">
-        <v>162</v>
+        <v>190</v>
       </c>
     </row>
     <row r="33" spans="1:18">
       <c r="A33" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B33" t="s">
         <v>54</v>
       </c>
       <c r="C33" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D33" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F33" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G33" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H33">
-        <v>0.28</v>
+        <v>2.2511</v>
       </c>
       <c r="I33" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="J33" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K33" s="2">
-        <v>46036.3125</v>
+        <v>46035.61805555555</v>
       </c>
       <c r="L33">
         <v>90</v>
       </c>
       <c r="M33" s="2">
-        <v>46036.375</v>
+        <v>46035.68055555555</v>
       </c>
       <c r="N33">
-        <v>3211</v>
+        <v>4110</v>
       </c>
       <c r="O33" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="P33" s="2">
-        <v>46038.60486111111</v>
+        <v>46038.53472222222</v>
       </c>
       <c r="Q33" s="2">
-        <v>46039.42569444444</v>
+        <v>46038.59513888889</v>
       </c>
       <c r="R33" t="s">
-        <v>161</v>
+        <v>188</v>
       </c>
     </row>
     <row r="34" spans="1:18">
@@ -3273,108 +3351,108 @@
         <v>55</v>
       </c>
       <c r="C34" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D34" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E34" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F34" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="G34" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H34">
-        <v>2.2733</v>
+        <v>2.2511</v>
       </c>
       <c r="I34" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J34" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K34" s="2">
-        <v>46036.41666666666</v>
+        <v>46035.69444444445</v>
       </c>
       <c r="L34">
         <v>90</v>
       </c>
       <c r="M34" s="2">
-        <v>46036.47916666666</v>
+        <v>46035.75694444445</v>
       </c>
       <c r="N34">
-        <v>2101</v>
+        <v>4087</v>
       </c>
       <c r="O34" t="s">
-        <v>156</v>
+        <v>184</v>
       </c>
       <c r="P34" s="2">
-        <v>46037.93819444445</v>
+        <v>46038.59513888889</v>
       </c>
       <c r="Q34" s="2">
-        <v>46038.38055555556</v>
+        <v>46038.65555555555</v>
       </c>
       <c r="R34" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="35" spans="1:18">
       <c r="A35" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B35" t="s">
         <v>56</v>
       </c>
       <c r="C35" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D35" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F35" t="s">
-        <v>141</v>
+        <v>73</v>
       </c>
       <c r="G35" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H35">
-        <v>2.2511</v>
+        <v>2.2948</v>
       </c>
       <c r="I35" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J35" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K35" s="2">
-        <v>46036.49305555555</v>
+        <v>46035.71527777778</v>
       </c>
       <c r="L35">
         <v>90</v>
       </c>
       <c r="M35" s="2">
-        <v>46036.55555555555</v>
+        <v>46035.77777777778</v>
       </c>
       <c r="N35">
-        <v>2850</v>
+        <v>1410</v>
       </c>
       <c r="O35" t="s">
-        <v>156</v>
+        <v>185</v>
       </c>
       <c r="P35" s="2">
-        <v>46038.53472222222</v>
+        <v>46036.75694444445</v>
       </c>
       <c r="Q35" s="2">
-        <v>46038.59513888889</v>
+        <v>46036.79861111111</v>
       </c>
       <c r="R35" t="s">
-        <v>160</v>
+        <v>188</v>
       </c>
     </row>
     <row r="36" spans="1:18">
@@ -3385,52 +3463,108 @@
         <v>57</v>
       </c>
       <c r="C36" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D36" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E36" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F36" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G36" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H36">
-        <v>2.2511</v>
+        <v>2.2544</v>
       </c>
       <c r="I36" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J36" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K36" s="2">
-        <v>46036.56944444445</v>
+        <v>46035.79166666666</v>
       </c>
       <c r="L36">
         <v>90</v>
       </c>
       <c r="M36" s="2">
-        <v>46036.63194444445</v>
+        <v>46035.85416666666</v>
       </c>
       <c r="N36">
-        <v>2827</v>
+        <v>2235</v>
       </c>
       <c r="O36" t="s">
-        <v>159</v>
+        <v>186</v>
       </c>
       <c r="P36" s="2">
-        <v>46038.59513888889</v>
+        <v>46037.40625</v>
       </c>
       <c r="Q36" s="2">
-        <v>46038.65555555555</v>
+        <v>46037.50069444445</v>
       </c>
       <c r="R36" t="s">
-        <v>160</v>
+        <v>188</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18">
+      <c r="A37" t="s">
+        <v>22</v>
+      </c>
+      <c r="B37" t="s">
+        <v>58</v>
+      </c>
+      <c r="C37" t="s">
+        <v>73</v>
+      </c>
+      <c r="D37" t="s">
+        <v>94</v>
+      </c>
+      <c r="E37" t="s">
+        <v>136</v>
+      </c>
+      <c r="F37" t="s">
+        <v>73</v>
+      </c>
+      <c r="G37" t="s">
+        <v>151</v>
+      </c>
+      <c r="H37">
+        <v>2.2948</v>
+      </c>
+      <c r="I37" t="s">
+        <v>152</v>
+      </c>
+      <c r="J37" t="s">
+        <v>154</v>
+      </c>
+      <c r="K37" s="2">
+        <v>46035.86805555555</v>
+      </c>
+      <c r="L37">
+        <v>90</v>
+      </c>
+      <c r="M37" s="2">
+        <v>46035.93055555555</v>
+      </c>
+      <c r="N37">
+        <v>2202</v>
+      </c>
+      <c r="O37" t="s">
+        <v>187</v>
+      </c>
+      <c r="P37" s="2">
+        <v>46037.45972222222</v>
+      </c>
+      <c r="Q37" s="2">
+        <v>46037.50138888889</v>
+      </c>
+      <c r="R37" t="s">
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -3440,1322 +3574,1280 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E144"/>
+  <dimension ref="A1:E145"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>163</v>
+        <v>191</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>164</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>165</v>
+        <v>193</v>
       </c>
       <c r="B2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D2" t="s">
-        <v>333</v>
+        <v>361</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>166</v>
+        <v>194</v>
       </c>
       <c r="B3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D3" t="s">
-        <v>333</v>
+        <v>362</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>167</v>
+        <v>195</v>
       </c>
       <c r="B4" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D4" t="s">
-        <v>333</v>
+        <v>362</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>168</v>
+        <v>196</v>
       </c>
       <c r="B5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D5" t="s">
-        <v>334</v>
+        <v>363</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>169</v>
+        <v>197</v>
       </c>
       <c r="B6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D6" t="s">
-        <v>334</v>
+        <v>363</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>170</v>
+        <v>198</v>
       </c>
       <c r="B7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D7" t="s">
-        <v>335</v>
+        <v>363</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>171</v>
+        <v>199</v>
       </c>
       <c r="B8" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D8" t="s">
-        <v>335</v>
+        <v>364</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>172</v>
+        <v>200</v>
       </c>
       <c r="B9" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D9" t="s">
-        <v>335</v>
+        <v>364</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>173</v>
+        <v>201</v>
       </c>
       <c r="B10" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D10" t="s">
-        <v>320</v>
+        <v>364</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>174</v>
+        <v>202</v>
       </c>
       <c r="B11" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D11" t="s">
-        <v>336</v>
+        <v>363</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>175</v>
+        <v>203</v>
       </c>
       <c r="B12" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D12" t="s">
-        <v>336</v>
+        <v>363</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>176</v>
+        <v>204</v>
       </c>
       <c r="B13" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D13" t="s">
-        <v>336</v>
+        <v>365</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>177</v>
+        <v>205</v>
       </c>
       <c r="B14" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D14" t="s">
-        <v>337</v>
+        <v>365</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>178</v>
+        <v>206</v>
       </c>
       <c r="B15" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D15" t="s">
-        <v>337</v>
+        <v>366</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>179</v>
+        <v>207</v>
       </c>
       <c r="B16" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D16" t="s">
-        <v>337</v>
+        <v>366</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>180</v>
+        <v>208</v>
       </c>
       <c r="B17" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D17" t="s">
-        <v>320</v>
+        <v>367</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>181</v>
+        <v>209</v>
       </c>
       <c r="B18" t="s">
         <v>154</v>
       </c>
       <c r="D18" t="s">
-        <v>338</v>
+        <v>367</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>182</v>
+        <v>210</v>
       </c>
       <c r="B19" t="s">
         <v>154</v>
       </c>
       <c r="D19" t="s">
-        <v>338</v>
+        <v>367</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>183</v>
+        <v>211</v>
       </c>
       <c r="B20" t="s">
         <v>154</v>
       </c>
       <c r="D20" t="s">
-        <v>338</v>
+        <v>366</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>184</v>
+        <v>212</v>
       </c>
       <c r="B21" t="s">
         <v>154</v>
       </c>
       <c r="D21" t="s">
-        <v>339</v>
+        <v>363</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
-        <v>185</v>
+        <v>213</v>
       </c>
       <c r="B22" t="s">
         <v>154</v>
       </c>
+      <c r="C22" t="s">
+        <v>337</v>
+      </c>
       <c r="D22" t="s">
-        <v>339</v>
+        <v>368</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>186</v>
+        <v>214</v>
       </c>
       <c r="B23" t="s">
         <v>154</v>
       </c>
+      <c r="C23" t="s">
+        <v>337</v>
+      </c>
       <c r="D23" t="s">
-        <v>339</v>
+        <v>368</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>187</v>
+        <v>215</v>
       </c>
       <c r="B24" t="s">
         <v>154</v>
       </c>
+      <c r="C24" t="s">
+        <v>337</v>
+      </c>
       <c r="D24" t="s">
-        <v>320</v>
+        <v>368</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>188</v>
+        <v>216</v>
       </c>
       <c r="B25" t="s">
         <v>154</v>
+      </c>
+      <c r="C25" t="s">
+        <v>338</v>
+      </c>
+      <c r="D25" t="s">
+        <v>369</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>189</v>
+        <v>217</v>
       </c>
       <c r="B26" t="s">
         <v>154</v>
       </c>
+      <c r="C26" t="s">
+        <v>338</v>
+      </c>
       <c r="D26" t="s">
-        <v>340</v>
+        <v>369</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>190</v>
+        <v>218</v>
       </c>
       <c r="B27" t="s">
         <v>154</v>
       </c>
+      <c r="C27" t="s">
+        <v>338</v>
+      </c>
       <c r="D27" t="s">
-        <v>340</v>
+        <v>369</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>191</v>
+        <v>219</v>
       </c>
       <c r="B28" t="s">
         <v>154</v>
       </c>
+      <c r="C28" t="s">
+        <v>339</v>
+      </c>
       <c r="D28" t="s">
-        <v>340</v>
+        <v>366</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>192</v>
+        <v>220</v>
       </c>
       <c r="B29" t="s">
         <v>154</v>
       </c>
+      <c r="C29" t="s">
+        <v>339</v>
+      </c>
       <c r="D29" t="s">
-        <v>334</v>
+        <v>370</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>193</v>
+        <v>221</v>
       </c>
       <c r="B30" t="s">
         <v>154</v>
       </c>
+      <c r="C30" t="s">
+        <v>339</v>
+      </c>
       <c r="D30" t="s">
-        <v>334</v>
+        <v>370</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>194</v>
+        <v>222</v>
       </c>
       <c r="B31" t="s">
         <v>154</v>
+      </c>
+      <c r="C31" t="s">
+        <v>340</v>
+      </c>
+      <c r="D31" t="s">
+        <v>370</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" t="s">
-        <v>195</v>
+        <v>223</v>
       </c>
       <c r="B32" t="s">
         <v>154</v>
+      </c>
+      <c r="C32" t="s">
+        <v>340</v>
+      </c>
+      <c r="D32" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>196</v>
+        <v>224</v>
       </c>
       <c r="B33" t="s">
-        <v>152</v>
+        <v>154</v>
+      </c>
+      <c r="C33" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>197</v>
+        <v>225</v>
       </c>
       <c r="B34" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>198</v>
+        <v>226</v>
       </c>
       <c r="B35" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>199</v>
+        <v>227</v>
       </c>
       <c r="B36" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>200</v>
+        <v>228</v>
       </c>
       <c r="B37" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>201</v>
+        <v>229</v>
       </c>
       <c r="B38" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>202</v>
+        <v>230</v>
       </c>
       <c r="B39" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>203</v>
+        <v>231</v>
       </c>
       <c r="B40" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>204</v>
+        <v>232</v>
       </c>
       <c r="B41" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>205</v>
+        <v>233</v>
       </c>
       <c r="B42" t="s">
-        <v>152</v>
-      </c>
-      <c r="C42" t="s">
-        <v>308</v>
+        <v>156</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>206</v>
+        <v>234</v>
       </c>
       <c r="B43" t="s">
-        <v>152</v>
-      </c>
-      <c r="C43" t="s">
-        <v>308</v>
+        <v>156</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>207</v>
+        <v>235</v>
       </c>
       <c r="B44" t="s">
-        <v>152</v>
-      </c>
-      <c r="C44" t="s">
-        <v>308</v>
+        <v>156</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>208</v>
+        <v>236</v>
       </c>
       <c r="B45" t="s">
-        <v>152</v>
-      </c>
-      <c r="C45" t="s">
-        <v>309</v>
+        <v>156</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>209</v>
+        <v>237</v>
       </c>
       <c r="B46" t="s">
-        <v>152</v>
-      </c>
-      <c r="C46" t="s">
-        <v>309</v>
+        <v>156</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>210</v>
+        <v>238</v>
       </c>
       <c r="B47" t="s">
-        <v>152</v>
-      </c>
-      <c r="C47" t="s">
-        <v>309</v>
+        <v>156</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>211</v>
+        <v>239</v>
       </c>
       <c r="B48" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>212</v>
+        <v>240</v>
       </c>
       <c r="B49" t="s">
-        <v>153</v>
-      </c>
-      <c r="D49" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" t="s">
+        <v>241</v>
+      </c>
+      <c r="B50" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" t="s">
+        <v>242</v>
+      </c>
+      <c r="B51" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" t="s">
+        <v>243</v>
+      </c>
+      <c r="B52" t="s">
+        <v>155</v>
+      </c>
+      <c r="C52" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
-      <c r="A50" t="s">
-        <v>213</v>
-      </c>
-      <c r="B50" t="s">
-        <v>153</v>
-      </c>
-      <c r="D50" t="s">
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
+        <v>244</v>
+      </c>
+      <c r="B53" t="s">
+        <v>155</v>
+      </c>
+      <c r="C53" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="51" spans="1:4">
-      <c r="A51" t="s">
-        <v>214</v>
-      </c>
-      <c r="B51" t="s">
-        <v>153</v>
-      </c>
-      <c r="D51" t="s">
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
+        <v>245</v>
+      </c>
+      <c r="B54" t="s">
+        <v>155</v>
+      </c>
+      <c r="C54" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="52" spans="1:4">
-      <c r="A52" t="s">
-        <v>215</v>
-      </c>
-      <c r="B52" t="s">
-        <v>153</v>
-      </c>
-      <c r="C52" t="s">
-        <v>310</v>
-      </c>
-      <c r="D52" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4">
-      <c r="A53" t="s">
-        <v>216</v>
-      </c>
-      <c r="B53" t="s">
-        <v>153</v>
-      </c>
-      <c r="C53" t="s">
-        <v>310</v>
-      </c>
-      <c r="D53" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4">
-      <c r="A54" t="s">
-        <v>217</v>
-      </c>
-      <c r="B54" t="s">
-        <v>153</v>
-      </c>
-      <c r="C54" t="s">
-        <v>310</v>
-      </c>
-      <c r="D54" t="s">
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
+        <v>246</v>
+      </c>
+      <c r="B55" t="s">
+        <v>155</v>
+      </c>
+      <c r="C55" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="55" spans="1:4">
-      <c r="A55" t="s">
-        <v>218</v>
-      </c>
-      <c r="B55" t="s">
-        <v>153</v>
-      </c>
-      <c r="C55" t="s">
-        <v>311</v>
-      </c>
-      <c r="D55" t="s">
+    <row r="56" spans="1:3">
+      <c r="A56" t="s">
+        <v>247</v>
+      </c>
+      <c r="B56" t="s">
+        <v>155</v>
+      </c>
+      <c r="C56" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
-      <c r="A56" t="s">
-        <v>219</v>
-      </c>
-      <c r="B56" t="s">
-        <v>153</v>
-      </c>
-      <c r="C56" t="s">
-        <v>311</v>
-      </c>
-      <c r="D56" t="s">
+    <row r="57" spans="1:3">
+      <c r="A57" t="s">
+        <v>248</v>
+      </c>
+      <c r="B57" t="s">
+        <v>155</v>
+      </c>
+      <c r="C57" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="57" spans="1:4">
-      <c r="A57" t="s">
-        <v>220</v>
-      </c>
-      <c r="B57" t="s">
-        <v>153</v>
-      </c>
-      <c r="C57" t="s">
-        <v>311</v>
-      </c>
-      <c r="D57" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4">
+    <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>221</v>
+        <v>249</v>
       </c>
       <c r="B58" t="s">
-        <v>153</v>
-      </c>
-      <c r="D58" t="s">
+        <v>155</v>
+      </c>
+      <c r="C58" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="59" spans="1:4">
+    <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>222</v>
+        <v>250</v>
       </c>
       <c r="B59" t="s">
-        <v>153</v>
-      </c>
-      <c r="D59" t="s">
+        <v>155</v>
+      </c>
+      <c r="C59" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="60" spans="1:4">
+    <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>223</v>
+        <v>251</v>
       </c>
       <c r="B60" t="s">
-        <v>153</v>
-      </c>
-      <c r="D60" t="s">
+        <v>155</v>
+      </c>
+      <c r="C60" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="61" spans="1:4">
+    <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>224</v>
+        <v>252</v>
       </c>
       <c r="B61" t="s">
-        <v>153</v>
-      </c>
-      <c r="D61" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4">
+        <v>155</v>
+      </c>
+      <c r="C61" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>225</v>
+        <v>253</v>
       </c>
       <c r="B62" t="s">
-        <v>153</v>
-      </c>
-      <c r="D62" t="s">
+        <v>155</v>
+      </c>
+      <c r="C62" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="63" spans="1:4">
+    <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>226</v>
+        <v>254</v>
       </c>
       <c r="B63" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C63" t="s">
-        <v>312</v>
-      </c>
-      <c r="D63" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="64" spans="1:4">
+    <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>227</v>
+        <v>255</v>
       </c>
       <c r="B64" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C64" t="s">
-        <v>312</v>
-      </c>
-      <c r="D64" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>228</v>
+        <v>256</v>
       </c>
       <c r="B65" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C65" t="s">
-        <v>312</v>
+        <v>345</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>229</v>
+        <v>257</v>
       </c>
       <c r="B66" t="s">
         <v>154</v>
+      </c>
+      <c r="C66" t="s">
+        <v>345</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>230</v>
+        <v>258</v>
       </c>
       <c r="B67" t="s">
         <v>154</v>
       </c>
       <c r="C67" t="s">
-        <v>313</v>
+        <v>346</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>231</v>
+        <v>259</v>
       </c>
       <c r="B68" t="s">
         <v>154</v>
       </c>
       <c r="C68" t="s">
-        <v>313</v>
+        <v>346</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>232</v>
+        <v>260</v>
       </c>
       <c r="B69" t="s">
         <v>154</v>
       </c>
       <c r="C69" t="s">
-        <v>313</v>
+        <v>346</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>233</v>
+        <v>261</v>
       </c>
       <c r="B70" t="s">
         <v>154</v>
+      </c>
+      <c r="C70" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>234</v>
+        <v>262</v>
       </c>
       <c r="B71" t="s">
         <v>154</v>
+      </c>
+      <c r="C71" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>235</v>
+        <v>263</v>
       </c>
       <c r="B72" t="s">
         <v>154</v>
       </c>
       <c r="C72" t="s">
-        <v>314</v>
+        <v>347</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>236</v>
+        <v>264</v>
       </c>
       <c r="B73" t="s">
         <v>154</v>
       </c>
       <c r="C73" t="s">
-        <v>314</v>
+        <v>348</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>237</v>
+        <v>265</v>
       </c>
       <c r="B74" t="s">
         <v>154</v>
       </c>
       <c r="C74" t="s">
-        <v>314</v>
+        <v>348</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>238</v>
+        <v>266</v>
       </c>
       <c r="B75" t="s">
         <v>154</v>
       </c>
       <c r="C75" t="s">
-        <v>315</v>
+        <v>348</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>239</v>
+        <v>267</v>
       </c>
       <c r="B76" t="s">
         <v>154</v>
       </c>
       <c r="C76" t="s">
-        <v>315</v>
+        <v>349</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>240</v>
+        <v>268</v>
       </c>
       <c r="B77" t="s">
         <v>154</v>
       </c>
       <c r="C77" t="s">
-        <v>315</v>
+        <v>349</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>241</v>
+        <v>269</v>
       </c>
       <c r="B78" t="s">
         <v>154</v>
       </c>
       <c r="C78" t="s">
-        <v>316</v>
+        <v>349</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>242</v>
+        <v>270</v>
       </c>
       <c r="B79" t="s">
         <v>154</v>
       </c>
       <c r="C79" t="s">
-        <v>316</v>
+        <v>350</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>243</v>
+        <v>271</v>
       </c>
       <c r="B80" t="s">
         <v>154</v>
       </c>
       <c r="C80" t="s">
-        <v>316</v>
+        <v>350</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>244</v>
+        <v>272</v>
       </c>
       <c r="B81" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C81" t="s">
-        <v>317</v>
+        <v>350</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>245</v>
+        <v>273</v>
       </c>
       <c r="B82" t="s">
-        <v>152</v>
-      </c>
-      <c r="C82" t="s">
-        <v>317</v>
+        <v>156</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>246</v>
+        <v>274</v>
       </c>
       <c r="B83" t="s">
-        <v>152</v>
-      </c>
-      <c r="C83" t="s">
-        <v>317</v>
+        <v>156</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>247</v>
+        <v>275</v>
       </c>
       <c r="B84" t="s">
-        <v>152</v>
-      </c>
-      <c r="C84" t="s">
-        <v>318</v>
+        <v>156</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>248</v>
+        <v>276</v>
       </c>
       <c r="B85" t="s">
-        <v>152</v>
-      </c>
-      <c r="C85" t="s">
-        <v>318</v>
+        <v>156</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>249</v>
+        <v>277</v>
       </c>
       <c r="B86" t="s">
-        <v>152</v>
-      </c>
-      <c r="C86" t="s">
-        <v>318</v>
+        <v>156</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>250</v>
+        <v>278</v>
       </c>
       <c r="B87" t="s">
-        <v>152</v>
-      </c>
-      <c r="C87" t="s">
-        <v>319</v>
+        <v>156</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>251</v>
+        <v>279</v>
       </c>
       <c r="B88" t="s">
-        <v>152</v>
-      </c>
-      <c r="C88" t="s">
-        <v>319</v>
+        <v>156</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>252</v>
+        <v>280</v>
       </c>
       <c r="B89" t="s">
-        <v>152</v>
-      </c>
-      <c r="C89" t="s">
-        <v>319</v>
+        <v>156</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>253</v>
+        <v>281</v>
       </c>
       <c r="B90" t="s">
-        <v>152</v>
-      </c>
-      <c r="C90" t="s">
-        <v>320</v>
+        <v>156</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>254</v>
+        <v>282</v>
       </c>
       <c r="B91" t="s">
-        <v>152</v>
-      </c>
-      <c r="C91" t="s">
-        <v>321</v>
+        <v>156</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>255</v>
+        <v>283</v>
       </c>
       <c r="B92" t="s">
-        <v>152</v>
-      </c>
-      <c r="C92" t="s">
-        <v>321</v>
+        <v>156</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>256</v>
+        <v>284</v>
       </c>
       <c r="B93" t="s">
-        <v>152</v>
-      </c>
-      <c r="C93" t="s">
-        <v>321</v>
+        <v>156</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>257</v>
+        <v>285</v>
       </c>
       <c r="B94" t="s">
-        <v>152</v>
-      </c>
-      <c r="C94" t="s">
-        <v>322</v>
+        <v>156</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>258</v>
+        <v>286</v>
       </c>
       <c r="B95" t="s">
-        <v>152</v>
-      </c>
-      <c r="C95" t="s">
-        <v>322</v>
+        <v>156</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>259</v>
+        <v>287</v>
       </c>
       <c r="B96" t="s">
-        <v>152</v>
-      </c>
-      <c r="C96" t="s">
-        <v>322</v>
+        <v>156</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>260</v>
+        <v>288</v>
       </c>
       <c r="B97" t="s">
-        <v>153</v>
-      </c>
-      <c r="C97" t="s">
-        <v>323</v>
+        <v>156</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>261</v>
+        <v>289</v>
       </c>
       <c r="B98" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C98" t="s">
-        <v>323</v>
+        <v>351</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>262</v>
+        <v>290</v>
       </c>
       <c r="B99" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C99" t="s">
-        <v>323</v>
+        <v>351</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>263</v>
+        <v>291</v>
       </c>
       <c r="B100" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C100" t="s">
-        <v>324</v>
+        <v>351</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>264</v>
+        <v>292</v>
       </c>
       <c r="B101" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C101" t="s">
-        <v>324</v>
+        <v>352</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>265</v>
+        <v>293</v>
       </c>
       <c r="B102" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C102" t="s">
-        <v>324</v>
+        <v>352</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>266</v>
+        <v>294</v>
       </c>
       <c r="B103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C103" t="s">
-        <v>325</v>
+        <v>352</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>267</v>
+        <v>295</v>
       </c>
       <c r="B104" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C104" t="s">
-        <v>325</v>
+        <v>353</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>268</v>
+        <v>296</v>
       </c>
       <c r="B105" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C105" t="s">
-        <v>325</v>
+        <v>353</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>269</v>
+        <v>297</v>
       </c>
       <c r="B106" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C106" t="s">
-        <v>326</v>
+        <v>353</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>270</v>
+        <v>298</v>
       </c>
       <c r="B107" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C107" t="s">
-        <v>326</v>
+        <v>354</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>271</v>
+        <v>299</v>
       </c>
       <c r="B108" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C108" t="s">
-        <v>326</v>
+        <v>354</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>272</v>
+        <v>300</v>
       </c>
       <c r="B109" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C109" t="s">
-        <v>327</v>
+        <v>354</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>273</v>
+        <v>301</v>
       </c>
       <c r="B110" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C110" t="s">
-        <v>327</v>
+        <v>355</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>274</v>
+        <v>302</v>
       </c>
       <c r="B111" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C111" t="s">
-        <v>327</v>
+        <v>355</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>275</v>
+        <v>303</v>
       </c>
       <c r="B112" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C112" t="s">
-        <v>328</v>
+        <v>355</v>
       </c>
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>276</v>
+        <v>304</v>
       </c>
       <c r="B113" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C113" t="s">
-        <v>328</v>
+        <v>356</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>277</v>
+        <v>305</v>
       </c>
       <c r="B114" t="s">
         <v>154</v>
       </c>
       <c r="C114" t="s">
-        <v>328</v>
+        <v>356</v>
       </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>278</v>
+        <v>306</v>
       </c>
       <c r="B115" t="s">
         <v>154</v>
       </c>
       <c r="C115" t="s">
-        <v>329</v>
+        <v>356</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>279</v>
+        <v>307</v>
       </c>
       <c r="B116" t="s">
         <v>154</v>
       </c>
       <c r="C116" t="s">
-        <v>329</v>
+        <v>357</v>
       </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>280</v>
+        <v>308</v>
       </c>
       <c r="B117" t="s">
         <v>154</v>
       </c>
       <c r="C117" t="s">
-        <v>329</v>
+        <v>357</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>281</v>
+        <v>309</v>
       </c>
       <c r="B118" t="s">
         <v>154</v>
       </c>
       <c r="C118" t="s">
-        <v>330</v>
+        <v>357</v>
       </c>
     </row>
     <row r="119" spans="1:3">
       <c r="A119" t="s">
-        <v>282</v>
+        <v>310</v>
       </c>
       <c r="B119" t="s">
         <v>154</v>
       </c>
       <c r="C119" t="s">
-        <v>330</v>
+        <v>358</v>
       </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
-        <v>283</v>
+        <v>311</v>
       </c>
       <c r="B120" t="s">
         <v>154</v>
       </c>
       <c r="C120" t="s">
-        <v>330</v>
+        <v>358</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>284</v>
+        <v>312</v>
       </c>
       <c r="B121" t="s">
         <v>154</v>
+      </c>
+      <c r="C121" t="s">
+        <v>358</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>285</v>
+        <v>313</v>
       </c>
       <c r="B122" t="s">
         <v>154</v>
@@ -4763,7 +4855,7 @@
     </row>
     <row r="123" spans="1:3">
       <c r="A123" t="s">
-        <v>286</v>
+        <v>314</v>
       </c>
       <c r="B123" t="s">
         <v>154</v>
@@ -4771,7 +4863,7 @@
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>287</v>
+        <v>315</v>
       </c>
       <c r="B124" t="s">
         <v>154</v>
@@ -4779,180 +4871,188 @@
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>288</v>
+        <v>316</v>
       </c>
       <c r="B125" t="s">
         <v>154</v>
-      </c>
-      <c r="C125" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
-        <v>289</v>
+        <v>317</v>
       </c>
       <c r="B126" t="s">
         <v>154</v>
       </c>
       <c r="C126" t="s">
-        <v>331</v>
+        <v>359</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>290</v>
+        <v>318</v>
       </c>
       <c r="B127" t="s">
         <v>154</v>
       </c>
       <c r="C127" t="s">
-        <v>331</v>
+        <v>359</v>
       </c>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" t="s">
-        <v>291</v>
+        <v>319</v>
       </c>
       <c r="B128" t="s">
         <v>154</v>
+      </c>
+      <c r="C128" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>292</v>
+        <v>320</v>
       </c>
       <c r="B129" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>293</v>
+        <v>321</v>
       </c>
       <c r="B130" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>294</v>
+        <v>322</v>
       </c>
       <c r="B131" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>295</v>
+        <v>323</v>
       </c>
       <c r="B132" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>296</v>
+        <v>324</v>
       </c>
       <c r="B133" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
-        <v>297</v>
+        <v>325</v>
       </c>
       <c r="B134" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>298</v>
+        <v>326</v>
       </c>
       <c r="B135" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>299</v>
+        <v>327</v>
       </c>
       <c r="B136" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>300</v>
+        <v>328</v>
       </c>
       <c r="B137" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="138" spans="1:3">
       <c r="A138" t="s">
-        <v>301</v>
+        <v>329</v>
       </c>
       <c r="B138" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>302</v>
+        <v>330</v>
       </c>
       <c r="B139" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="140" spans="1:3">
       <c r="A140" t="s">
-        <v>303</v>
+        <v>331</v>
       </c>
       <c r="B140" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
-        <v>304</v>
+        <v>332</v>
       </c>
       <c r="B141" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>305</v>
+        <v>333</v>
       </c>
       <c r="B142" t="s">
-        <v>152</v>
-      </c>
-      <c r="C142" t="s">
-        <v>332</v>
+        <v>156</v>
       </c>
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>306</v>
+        <v>334</v>
       </c>
       <c r="B143" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C143" t="s">
-        <v>332</v>
+        <v>360</v>
       </c>
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>307</v>
+        <v>335</v>
       </c>
       <c r="B144" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C144" t="s">
-        <v>332</v>
+        <v>360</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3">
+      <c r="A145" t="s">
+        <v>336</v>
+      </c>
+      <c r="B145" t="s">
+        <v>156</v>
+      </c>
+      <c r="C145" t="s">
+        <v>360</v>
       </c>
     </row>
   </sheetData>

</xml_diff>